<commit_message>
Update README and test automation script for transliteration testing
- Revised the note on script adaptation in README to clarify the use of alternative URL for testing.
- Updated the default frontend URL in the test automation script to the official Chat Sinhala transliteration application.
- Enhanced code readability by formatting lists and improving variable names in the test automation script.
- Adjusted timeout and retry settings for better performance during tests.
</commit_message>
<xml_diff>
--- a/IT23192850.xlsx
+++ b/IT23192850.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>අපි ගූගල් මීට් එකෙන් කෝල් එකක් ගන්නවා, ඔයා ජොයින් වෙනවද?</t>
+          <t>අපි Google Meet එකෙන් call එකක් ගන්නවා, ඔයා ජොයින් වෙනවද?</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>මචං මට අද ක්ලාස් එකට එන්න බැරි උනා, සර්ට මැසේජ් එකක් දාන්න පුලුවන්ද?</t>
+          <t>මචන් මට අද class එකට එන්න බැරි වුණා, සර්ට msg එකක් දාන්න පුළුවන්ද?</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>හෙට ඉන්ටර්විව් එක 2:00PM ට, පරක්කු වෙන්න එපා හොඳේ බන්.</t>
+          <t>හෙට intrview එක 2:00PM ට, පර්ක්කු වෙන්න එපා හොඳේ බන්.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>මචං, මාකට් කරන්න එපා දැන්...</t>
+          <t>මචන්, මොකට කරන්න එපා දැන්...</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>සුභ අවුරුද්දක් වේවා! උඹ පොඩ්ඩක් ලඟින් හිටපන්.</t>
+          <t>සුභ අවුරුද්දක් වේවා! උඹ පොඩ්ඩක් ලඟින් හිටපං.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>අයියේ ඔයාට ජය වේවා, exam එක හොඳට කරගන්න ලැබේවා!</t>
+          <t>අයියේ ඔයාට ජය වේවා, exam එක හොදට කරගන්න ලැබේවා!</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>කරුණාකරල පොත මට දෙන්න, මම චෙක් කරන්නන්.</t>
+          <t>කරුණාකරලා පොත මට දෙන්න, මම check කරන්නං.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>තාත්තා කිව්වා අපි අද රෑ 8ට ගෙදර එන්න ඕනි කියලා.</t>
+          <t>තාත්තා කිව්වා අපි අද රාත්‍රි 8ට ගෙදර එන්න ඕනි කියලා.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>අයියෝ නෑ බං, මම දන්නෙ නෑ.</t>
+          <t>අයියෝ නෑ බුන්ග්, මම දන්නෑ නේ.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>අනේ, හරි තමයි, මම දැන්ම බලන්නම් ඔයා කිව්ව දේ.</t>
+          <t>අනේ, හරි තමා, මම දැන්ම බලන්නං ඔයා කිව්වාදේ.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>හරි හරි මම ටිකක් පස්සෙ එන්නම් බන්</t>
+          <t>හරි හරි මම ටිකක් පස්සේ එන්නම් බන්</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>ටික ටික බලාගෙන යන්න නැත්නම් වරදෙන්න පුළුවන්.</t>
+          <t>ටික ටික බලාගෙන යන්න නැත්නම් වරදෙන්න පුළුවන්</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>විස්තර ටික nadun@gmail.com ට එවන්න.</t>
+          <t>details ටික nadun@gmail.කොම්ටා එවන්න.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>අයියෝ! මම මේක කරන්න ගියා... හරියන්නෙ නෑ නේද?</t>
+          <t>අයියෝ! මම මේක කරන්න ගියා... හරියන්න නෑ නේ ද?</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>මොකද්ද ඔයාගෙ නම</t>
+          <t>මොකද ඔයාගේ නම්</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>මං ඔයාට පස්සෙ කතා කරන්නම්, මතක තියාගන්න.</t>
+          <t>මන් ඔයාට පස්සේ කතා කරන්නම්, මතක තියාගන්න.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>මට ඔයාගේ ඊමේල් එකට CV එක යවන්න බැරි උනා.</t>
+          <t>මට ඔයාගේ email එකට CV ඒක යවන්නද බැරි උනා</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>ඔයා ටිකට් එක බුක් කරාද මං වෙනුවෙන්?</t>
+          <t>ඔය ticket එක book කරාද මං වෙනුවෙන්?</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>මම මීටින් එකේ ඉන්නවා, පස්සෙ කෝල් කරන්න බන්.</t>
+          <t>මම meeting එකේ ඉන්නවා, call me back later බන්.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>අපි ඔන් ද වේ ඉන්නවා, ටිකක් ඉස්සරහට එන්නම් බන්.</t>
+          <t>අපි on the way ඉන්නවා, ටිකක් ඉස්සරහට එන්නම් බන්</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>මම ෆයිල් එක අප්ලෝඩ් කරන්න ට්‍රයි කළා, ඒත් සර්වර් එක එරර් දුන්නා.</t>
+          <t>මම file එක upload කරන්න try කළා, ඒත් server එක error දුන්.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>ඔයා මගේ ඊමේල් එක චෙක් කරාද, ඇටෑච්මන්ට් එක ආව නිසා ඉන්න ඕනි.</t>
+          <t>ඔයා මගේ email එක check කරාද, attachment එක ආවා නිසා ඉන්න ඕනේ.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>මම ඉන්ස්ටග්‍රෑම් ස්ටෝරි දාපු එක, ඔයා බැලුවද?</t>
+          <t>මම Instagram story දාපු එක, ඔයා බලලාද?</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>අපි වට්ස්ඇප් එකෙන් මැසේජ් එකක් යවන්න හිතුවා, ඒත් මම දැන්ම සෙන්ඩ් කරන්න බැරි උනා.</t>
+          <t>අපි WhatsApp ඒකෙන් msg එකක් යන්න හිතුවා, ඒත් මම දැන්ම send කරන්න බැරි වුණා.</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>ඔයා මගේ CV එක බලලා දන්නවද, OK ද?</t>
+          <t>ඔයා මගේ CV ඒක බලලා දන්නවද, OK ද?</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>FYI මම හෙට ඔෆිස් එන්නේ නෑ, WFH කරනවා.</t>
+          <t>FYI මම හෙට office එනවා, WFH කරනවා.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>මම අද ජිම් එක ගියා, සුපර් ටයර්ඩ් ඩන්ග්.</t>
+          <t>මම අද gym එක ගියා, සුපර් ටිරේඩ් ඩන්ග්.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>යුනි එකේ සබ් එක ෆේල් උනත් රී-සිට් දෙන්නවද?</t>
+          <t>උනි එකේ sub එක fail උනත් re-sit දෙන්නවද?</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>මම නෙක්ස්ට් වීක් නුවර එළිය යනවා, ඔයා එනවද?</t>
+          <t>මම next week නුවර එළිය යනවා, ඔයා එනවද?</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>අපි එල්ල ට්‍රිප් එකක් යන්න ප්ලෑන් කළා, එහේ විව් එක ලස්සනයි කියලා කියන්න නිසා.</t>
+          <t>අපි එල trip එකක් යන්න plan කළා, එහේ view එක ලස්සනයි කියලා කියන්න නිසා.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>නිමල් අය්යා කිව්වා මම හෙට ලේට් එන්නම් කියලා.</t>
+          <t>නිමල් අයියා කිව්වා මම හෙට late එන්නම් කියලා.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>දිලානි සහ කමලා දෙන්නම එක්සෑම් පාස් උනා.</t>
+          <t>දිලානි සහ කමලා දෙන්නම exam pass වුණා.</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>මම 3වෙනි උත්සාහයේදී තමයි පාස් උනා.</t>
+          <t>මම 3rd atempt එකේ තමයි pass වුණා.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>අපි අද 15ක් විතර ගියා, ගොඩක් ටයර්ඩ්.</t>
+          <t>අපි අද 15ක් විතර ගියා, ගොඩක් tired.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>මම USD 45k ගෙව්වා, ඒත් රිසිට් එක ඇවිල්ල නෑ.</t>
+          <t>මම USD 45ක් pay කළා, ඒත්‍රෙසිප්ට් එක ඇවිල්ලා නේ.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>ඔයා රු. 500 එක පෙන්නන්නකෝ, මම දැන්ම ගන්නම්.</t>
+          <t>ඔය Rs. 500 ඒක පෙන්නන්නකෝ, මම දැන්ම ගන්නන්.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>පන්තිය උදේ 8.30ට පටන් ගන්නවා, පරක්කු වෙන්න එපා.</t>
+          <t>class එක 8.30AMට start වෙනවා, late වෙන්න එපා.</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>මීටිම එක 7:45PM ට පටන් ගන්න කියල සර් කිව්වා.</t>
+          <t>meeting එක 7:45PM ට පටන් ගන්න කියලා sir කිව්වා.</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>මගේ බර්ත්ඩේ එක මාර්තු 12ට, හැබැයි පාටි නෑ.</t>
+          <t>මගේ බ්ර්ත්ඩය් එක මාර්තු 12 ට, හැබැයි party නෑ.</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>ඊළඟ මීටිම 2026-04-10ට ෂෙඩියුල් කරලා.</t>
+          <t>next meeting එක 2026-04-10ට schedule කරලා.</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>මම හෙට 5km විතර දුවනවා, ට්‍රේනින් එකේ.</t>
+          <t>මම හෙට 5km වත්රා දුවනවා, training එකේ.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>මම 5kg වෙයිට් එකක් අඩු කරගත්තා, දැන් ෂේප් එක හරි.</t>
+          <t>මම 5kg weight එකක් අඩු කරගත්ත, දැන් shape එක හරි.</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>බන් ඔයාට කිව්වනේ, මම පස්සේ එන්නම් කියලා.</t>
+          <t>බන් ඔයාට කිව්වා නේ, මම පස්සේ එන්නම් කියලා.</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>මට මේ ලින්ක් එක එවන්න https://forms.google.com මං බලන්නම් පස්සෙ.</t>
+          <t>මට මේ link එක එවන්න https://ෆොර්ම්ස්.ගූගල්.කොම් මන් බලන්නම් පස්සේ</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>@කසුන් මම ඔයාට ඊමේල් එකක් යැව්වා, චෙක් කරපන්.</t>
+          <t>@කසුන් මම ඔයාට email එකක් යවල, චෙක් කරපන්ග්.</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>අඩෝ 😂 මම මේක කරන්න ට්‍රයි කළා, හරියන්නෙ නෑ 😭</t>
+          <t>අඩෝ 😂 මම මේක කරන්න try කළා, හරියන්න නෑ 😭</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>මාර කේස්😅 මට ප්‍රොජෙක්ට් එක සබ්මිට් කරන්න බැරි උනා, ලෙක්චරට කියන්නද මොකක්ද කරන්නෙ 😓</t>
+          <t>මාර case😅 මට project එක submit කරන්න බැරි වුණා, lecturer ට කියන්නද මොකක්ද කරන්නේ</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>අපි Zoom එකෙන් මීටිං එකක් ගන්න සෙට් කරන්න, ඔයා ජොයින් වෙනවද?</t>
+          <t>අපි Zoom ඒකෙන් meeting එකක් ගන්න set කරන්න, ඔයා join වෙනවද?</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>මම හෙට සුභ උත්සවයට යනවා, ඔයා එනවද? අපි එක්ක යමු. ගැදරින්ග් එක 6:00PM ට, කොළඹ 3 අර හෝටලේ. දිල්ෂාන් අය්යා කිව්වා RSVP කරන්න ඕනි කියලා. මට රු. 1500 එක ගොඩක් බඩු, ඔයා ෂෙයාර් කරනවද? 😊</t>
+          <t>මම හෙට සුභ උත්සවයට යනවා, ඔයා එනවද? අපි එක්ක යමු. gathering එක 6:00PM ට, Colombo 3 අර හොටෙල් එකේ. දිල්ෂාන් අයියා කිව්වා RSVP කරන්න ඕනි කියලා. මට Rs. 1500 ඒක ගොඩක් බඩු, ඔයා share කරනවද? 😊</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">

</xml_diff>